<commit_message>
Otomatik veri güncelleme (13.08.2026 12:33 UTC)
</commit_message>
<xml_diff>
--- a/cari acik/cari_acik_son.xlsx
+++ b/cari acik/cari_acik_son.xlsx
@@ -640,10 +640,10 @@
         <v>-10262</v>
       </c>
       <c r="C14" t="n">
-        <v>-5670</v>
+        <v>-5141</v>
       </c>
       <c r="D14" t="n">
-        <v>4613</v>
+        <v>5142</v>
       </c>
     </row>
     <row r="15">
@@ -656,10 +656,10 @@
         <v>-9574</v>
       </c>
       <c r="C15" t="n">
-        <v>-12636</v>
+        <v>-10840</v>
       </c>
       <c r="D15" t="n">
-        <v>-3059</v>
+        <v>-1263</v>
       </c>
     </row>
     <row r="16">
@@ -672,10 +672,10 @@
         <v>-482</v>
       </c>
       <c r="C16" t="n">
-        <v>-5292</v>
+        <v>-5304</v>
       </c>
       <c r="D16" t="n">
-        <v>-4767</v>
+        <v>-4779</v>
       </c>
     </row>
     <row r="17">
@@ -688,10 +688,10 @@
         <v>-11794</v>
       </c>
       <c r="C17" t="n">
-        <v>-15947</v>
+        <v>-15230</v>
       </c>
       <c r="D17" t="n">
-        <v>-4150</v>
+        <v>-3433</v>
       </c>
     </row>
     <row r="18">
@@ -704,10 +704,10 @@
         <v>-8554</v>
       </c>
       <c r="C18" t="n">
-        <v>-10545</v>
+        <v>-10499</v>
       </c>
       <c r="D18" t="n">
-        <v>-1990</v>
+        <v>-1944</v>
       </c>
     </row>
     <row r="19">
@@ -720,10 +720,10 @@
         <v>-8790</v>
       </c>
       <c r="C19" t="n">
-        <v>-4396</v>
+        <v>-5642</v>
       </c>
       <c r="D19" t="n">
-        <v>4394</v>
+        <v>3148</v>
       </c>
     </row>
     <row r="20">
@@ -736,10 +736,10 @@
         <v>2360</v>
       </c>
       <c r="C20" t="n">
-        <v>3061</v>
+        <v>884</v>
       </c>
       <c r="D20" t="n">
-        <v>706</v>
+        <v>-1471</v>
       </c>
     </row>
     <row r="21">
@@ -752,10 +752,10 @@
         <v>-6368</v>
       </c>
       <c r="C21" t="n">
-        <v>-6244</v>
+        <v>-5676</v>
       </c>
       <c r="D21" t="n">
-        <v>139</v>
+        <v>707</v>
       </c>
     </row>
     <row r="22">
@@ -768,10 +768,10 @@
         <v>-6604</v>
       </c>
       <c r="C22" t="n">
-        <v>-7056</v>
+        <v>-6599</v>
       </c>
       <c r="D22" t="n">
-        <v>-467</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="23">
@@ -784,10 +784,10 @@
         <v>-9155</v>
       </c>
       <c r="C23" t="n">
-        <v>-11261</v>
+        <v>-11150</v>
       </c>
       <c r="D23" t="n">
-        <v>-2106</v>
+        <v>-1995</v>
       </c>
     </row>
     <row r="24">
@@ -800,10 +800,10 @@
         <v>-784</v>
       </c>
       <c r="C24" t="n">
-        <v>-2773</v>
+        <v>-2881</v>
       </c>
       <c r="D24" t="n">
-        <v>-1996</v>
+        <v>-2104</v>
       </c>
     </row>
     <row r="25">
@@ -816,10 +816,10 @@
         <v>-5622</v>
       </c>
       <c r="C25" t="n">
-        <v>4366</v>
+        <v>2163</v>
       </c>
       <c r="D25" t="n">
-        <v>9988</v>
+        <v>7785</v>
       </c>
     </row>
     <row r="26">
@@ -832,10 +832,10 @@
         <v>-6985</v>
       </c>
       <c r="C26" t="n">
-        <v>-12368</v>
+        <v>-12037</v>
       </c>
       <c r="D26" t="n">
-        <v>-5371</v>
+        <v>-5040</v>
       </c>
     </row>
     <row r="27">
@@ -848,10 +848,10 @@
         <v>-10477</v>
       </c>
       <c r="C27" t="n">
-        <v>-12102</v>
+        <v>-10658</v>
       </c>
       <c r="D27" t="n">
-        <v>-1636</v>
+        <v>-192</v>
       </c>
     </row>
     <row r="28">
@@ -864,10 +864,10 @@
         <v>-4758</v>
       </c>
       <c r="C28" t="n">
-        <v>-12643</v>
+        <v>-11306</v>
       </c>
       <c r="D28" t="n">
-        <v>-7902</v>
+        <v>-6565</v>
       </c>
     </row>
     <row r="29">
@@ -880,10 +880,10 @@
         <v>-12921</v>
       </c>
       <c r="C29" t="n">
-        <v>-12552</v>
+        <v>-15126</v>
       </c>
       <c r="D29" t="n">
-        <v>370</v>
+        <v>-2204</v>
       </c>
     </row>
     <row r="30">
@@ -896,10 +896,10 @@
         <v>-15422</v>
       </c>
       <c r="C30" t="n">
-        <v>-10561</v>
+        <v>-10134</v>
       </c>
       <c r="D30" t="n">
-        <v>4825</v>
+        <v>5252</v>
       </c>
     </row>
     <row r="31">
@@ -912,10 +912,10 @@
         <v>-12973</v>
       </c>
       <c r="C31" t="n">
-        <v>-8150</v>
+        <v>-11662</v>
       </c>
       <c r="D31" t="n">
-        <v>4810</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="32">
@@ -928,10 +928,10 @@
         <v>7409</v>
       </c>
       <c r="C32" t="n">
-        <v>10791</v>
+        <v>8070</v>
       </c>
       <c r="D32" t="n">
-        <v>3352</v>
+        <v>631</v>
       </c>
     </row>
     <row r="33">
@@ -944,10 +944,10 @@
         <v>6378</v>
       </c>
       <c r="C33" t="n">
-        <v>9168</v>
+        <v>12811</v>
       </c>
       <c r="D33" t="n">
-        <v>2789</v>
+        <v>6432</v>
       </c>
     </row>
     <row r="34">
@@ -960,10 +960,10 @@
         <v>-305</v>
       </c>
       <c r="C34" t="n">
-        <v>-2104</v>
+        <v>-1059</v>
       </c>
       <c r="D34" t="n">
-        <v>-1825</v>
+        <v>-780</v>
       </c>
     </row>
     <row r="35">
@@ -976,10 +976,10 @@
         <v>1434</v>
       </c>
       <c r="C35" t="n">
-        <v>-63</v>
+        <v>-1091</v>
       </c>
       <c r="D35" t="n">
-        <v>-1489</v>
+        <v>-2517</v>
       </c>
     </row>
     <row r="36">
@@ -992,10 +992,10 @@
         <v>12723</v>
       </c>
       <c r="C36" t="n">
-        <v>7246</v>
+        <v>8783</v>
       </c>
       <c r="D36" t="n">
-        <v>-5497</v>
+        <v>-3960</v>
       </c>
     </row>
     <row r="37">
@@ -1008,10 +1008,10 @@
         <v>1161</v>
       </c>
       <c r="C37" t="n">
-        <v>248</v>
+        <v>501</v>
       </c>
       <c r="D37" t="n">
-        <v>-909</v>
+        <v>-656</v>
       </c>
     </row>
     <row r="38">
@@ -1024,10 +1024,10 @@
         <v>-6690</v>
       </c>
       <c r="C38" t="n">
-        <v>-12532</v>
+        <v>-13429</v>
       </c>
       <c r="D38" t="n">
-        <v>-5829</v>
+        <v>-6726</v>
       </c>
     </row>
     <row r="39">
@@ -1040,10 +1040,10 @@
         <v>-11110</v>
       </c>
       <c r="C39" t="n">
-        <v>-13840</v>
+        <v>-14090</v>
       </c>
       <c r="D39" t="n">
-        <v>-2723</v>
+        <v>-2973</v>
       </c>
     </row>
     <row r="40">
@@ -1056,10 +1056,10 @@
         <v>-6825</v>
       </c>
       <c r="C40" t="n">
-        <v>-9415</v>
+        <v>-8448</v>
       </c>
       <c r="D40" t="n">
-        <v>-2585</v>
+        <v>-1618</v>
       </c>
     </row>
     <row r="41">
@@ -1072,10 +1072,10 @@
         <v>-6399</v>
       </c>
       <c r="C41" t="n">
-        <v>-2959</v>
+        <v>-2424</v>
       </c>
       <c r="D41" t="n">
-        <v>3451</v>
+        <v>3986</v>
       </c>
     </row>
     <row r="42">
@@ -1088,10 +1088,10 @@
         <v>-6840</v>
       </c>
       <c r="C42" t="n">
-        <v>-2827</v>
+        <v>-5787</v>
       </c>
       <c r="D42" t="n">
-        <v>4034</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="43">
@@ -1104,10 +1104,10 @@
         <v>-5062</v>
       </c>
       <c r="C43" t="n">
-        <v>-1340</v>
+        <v>-4420</v>
       </c>
       <c r="D43" t="n">
-        <v>3720</v>
+        <v>640</v>
       </c>
     </row>
     <row r="44">
@@ -1120,10 +1120,10 @@
         <v>6508</v>
       </c>
       <c r="C44" t="n">
-        <v>14657</v>
+        <v>13208</v>
       </c>
       <c r="D44" t="n">
-        <v>8193</v>
+        <v>6744</v>
       </c>
     </row>
     <row r="45">
@@ -1136,10 +1136,10 @@
         <v>-1674</v>
       </c>
       <c r="C45" t="n">
-        <v>-7131</v>
+        <v>-8607</v>
       </c>
       <c r="D45" t="n">
-        <v>-5457</v>
+        <v>-6933</v>
       </c>
     </row>
     <row r="46">
@@ -1152,10 +1152,10 @@
         <v>-17956</v>
       </c>
       <c r="C46" t="n">
-        <v>-10222</v>
+        <v>-13138</v>
       </c>
       <c r="D46" t="n">
-        <v>7737</v>
+        <v>4821</v>
       </c>
     </row>
     <row r="47">
@@ -1168,10 +1168,10 @@
         <v>-11397</v>
       </c>
       <c r="C47" t="n">
-        <v>-3247</v>
+        <v>-6824</v>
       </c>
       <c r="D47" t="n">
-        <v>8161</v>
+        <v>4584</v>
       </c>
     </row>
     <row r="48">
@@ -1184,10 +1184,10 @@
         <v>-6448</v>
       </c>
       <c r="C48" t="n">
-        <v>-287</v>
+        <v>2114</v>
       </c>
       <c r="D48" t="n">
-        <v>6170</v>
+        <v>8571</v>
       </c>
     </row>
     <row r="49">
@@ -1200,10 +1200,10 @@
         <v>-10867</v>
       </c>
       <c r="C49" t="n">
-        <v>-5014</v>
+        <v>-5562</v>
       </c>
       <c r="D49" t="n">
-        <v>5865</v>
+        <v>5317</v>
       </c>
     </row>
     <row r="50">
@@ -1216,10 +1216,10 @@
         <v>-23976</v>
       </c>
       <c r="C50" t="n">
-        <v>-23500</v>
+        <v>-15462</v>
       </c>
       <c r="D50" t="n">
-        <v>523</v>
+        <v>8561</v>
       </c>
     </row>
     <row r="51">
@@ -1232,10 +1232,10 @@
         <v>-11193</v>
       </c>
       <c r="C51" t="n">
-        <v>-19257</v>
+        <v>-9534</v>
       </c>
       <c r="D51" t="n">
-        <v>-8027</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="52">
@@ -1248,10 +1248,10 @@
         <v>-2021</v>
       </c>
       <c r="C52" t="n">
-        <v>1312</v>
+        <v>-1677</v>
       </c>
       <c r="D52" t="n">
-        <v>3415</v>
+        <v>426</v>
       </c>
     </row>
     <row r="53">
@@ -1264,10 +1264,10 @@
         <v>-4631</v>
       </c>
       <c r="C53" t="n">
-        <v>-10455</v>
+        <v>-10726</v>
       </c>
       <c r="D53" t="n">
-        <v>-5786</v>
+        <v>-6057</v>
       </c>
     </row>
     <row r="54">
@@ -1280,10 +1280,10 @@
         <v>-9687</v>
       </c>
       <c r="C54" t="n">
-        <v>-17738</v>
+        <v>-13642</v>
       </c>
       <c r="D54" t="n">
-        <v>-8052</v>
+        <v>-3956</v>
       </c>
     </row>
     <row r="55">
@@ -1296,10 +1296,10 @@
         <v>-5140</v>
       </c>
       <c r="C55" t="n">
-        <v>-1587</v>
+        <v>-3515</v>
       </c>
       <c r="D55" t="n">
-        <v>3582</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="56">
@@ -1312,10 +1312,10 @@
         <v>8367</v>
       </c>
       <c r="C56" t="n">
-        <v>7226</v>
+        <v>8323</v>
       </c>
       <c r="D56" t="n">
-        <v>-1058</v>
+        <v>39</v>
       </c>
     </row>
     <row r="57">
@@ -1328,10 +1328,10 @@
         <v>-6567</v>
       </c>
       <c r="C57" t="n">
-        <v>-11616</v>
+        <v>-12060</v>
       </c>
       <c r="D57" t="n">
-        <v>-5034</v>
+        <v>-5478</v>
       </c>
     </row>
     <row r="58">
@@ -1344,10 +1344,10 @@
         <v>-14178</v>
       </c>
       <c r="C58" t="n">
-        <v>-16375</v>
+        <v>-14306</v>
       </c>
       <c r="D58" t="n">
-        <v>-2217</v>
+        <v>-148</v>
       </c>
     </row>
     <row r="59">
@@ -1360,10 +1360,10 @@
         <v>-11820</v>
       </c>
       <c r="C59" t="n">
-        <v>-15548</v>
+        <v>-11932</v>
       </c>
       <c r="D59" t="n">
-        <v>-3703</v>
+        <v>-87</v>
       </c>
     </row>
     <row r="60">
@@ -1376,10 +1376,10 @@
         <v>6886</v>
       </c>
       <c r="C60" t="n">
-        <v>2946</v>
+        <v>8807</v>
       </c>
       <c r="D60" t="n">
-        <v>-3777</v>
+        <v>2084</v>
       </c>
     </row>
     <row r="61">
@@ -1389,13 +1389,13 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>-11224</v>
+        <v>-11226</v>
       </c>
       <c r="C61" t="n">
-        <v>-20320</v>
+        <v>-18984</v>
       </c>
       <c r="D61" t="n">
-        <v>-9123</v>
+        <v>-7785</v>
       </c>
     </row>
     <row r="62">
@@ -1405,13 +1405,13 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>-23604</v>
+        <v>-23633</v>
       </c>
       <c r="C62" t="n">
-        <v>-40234</v>
+        <v>-37818</v>
       </c>
       <c r="D62" t="n">
-        <v>-16556</v>
+        <v>-14111</v>
       </c>
     </row>
     <row r="63">
@@ -1421,13 +1421,13 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>-7075</v>
+        <v>-10915</v>
       </c>
       <c r="C63" t="n">
-        <v>-9013</v>
+        <v>-11568</v>
       </c>
       <c r="D63" t="n">
-        <v>-1922</v>
+        <v>-624</v>
       </c>
     </row>
   </sheetData>

</xml_diff>